<commit_message>
test (similarity): Add filtering on Num article to integration test
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_similarities_body.xlsx
+++ b/tests/integration/test_data/test_similarities_body.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10112"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB768640-9842-5542-BD87-D7C181636F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6EFAEE4-A606-6B44-9DCB-9F717B38196E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="34400" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vieux amendements" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="40">
   <si>
     <t>Num amdt</t>
   </si>
@@ -77,9 +77,6 @@
   </si>
   <si>
     <t>La réponse est la suivante : foo</t>
-  </si>
-  <si>
-    <t>Article add. ap. 2</t>
   </si>
   <si>
     <t>au debut de la premiere phrase du 2deg du de l'article l. 137-13 du code de la securite sociale, le taux : &lt;&lt; 20 % &gt;&gt; est remplace par le taux : &lt;&lt; 30 % &gt;&gt;</t>
@@ -159,6 +156,9 @@
   </si>
   <si>
     <t>DIFFERENT PROJECT</t>
+  </si>
+  <si>
+    <t>MAUVAIS ARTICLE</t>
   </si>
 </sst>
 </file>
@@ -540,11 +540,12 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1000"/>
+  <dimension ref="A1:AA1001"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16" style="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="12.6640625" style="18" customWidth="1"/>
+    <col min="2" max="3" width="12.6640625" style="18" customWidth="1"/>
+    <col min="4" max="4" width="19.1640625" style="18" customWidth="1"/>
     <col min="5" max="5" width="33.6640625" style="18" customWidth="1"/>
     <col min="6" max="6" width="33.6640625" style="22" customWidth="1"/>
     <col min="7" max="7" width="39.5" style="18" customWidth="1"/>
@@ -557,7 +558,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>0</v>
@@ -606,7 +607,7 @@
     </row>
     <row r="2" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="6">
         <v>1</v>
@@ -621,10 +622,10 @@
         <v>11</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H2" s="19" t="s">
         <v>12</v>
@@ -639,7 +640,7 @@
     </row>
     <row r="3" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="6">
         <v>2</v>
@@ -654,87 +655,87 @@
         <v>11</v>
       </c>
       <c r="F3" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="10" t="s">
-        <v>25</v>
-      </c>
       <c r="H3" s="19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>13</v>
       </c>
       <c r="J3" s="19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K3" s="20"/>
     </row>
     <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B4" s="6">
         <v>3</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="E4" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H4" s="19" t="s">
         <v>16</v>
       </c>
       <c r="I4" s="6"/>
       <c r="J4" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K4" s="20"/>
     </row>
     <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B5" s="6">
         <v>3</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="E5" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" s="19" t="s">
         <v>16</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B6" s="9">
         <v>4</v>
@@ -743,35 +744,54 @@
         <v>9</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>15</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H6" s="19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I6" s="6"/>
       <c r="J6" s="19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="9"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="19"/>
+      <c r="A7" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="9">
+        <v>5</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="19" t="s">
+        <v>33</v>
+      </c>
       <c r="I7" s="6"/>
-      <c r="J7" s="19"/>
+      <c r="J7" s="19" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="9"/>
@@ -851,13 +871,13 @@
       <c r="J14" s="19"/>
     </row>
     <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="15"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
       <c r="F15" s="14"/>
       <c r="G15" s="10"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="19"/>
       <c r="I15" s="6"/>
       <c r="J15" s="19"/>
     </row>
@@ -873,16 +893,15 @@
       <c r="J16" s="19"/>
     </row>
     <row r="17" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
       <c r="F17" s="14"/>
       <c r="G17" s="10"/>
-      <c r="H17" s="19"/>
+      <c r="H17" s="23"/>
       <c r="I17" s="6"/>
       <c r="J17" s="19"/>
-      <c r="K17" s="20"/>
     </row>
     <row r="18" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="6"/>
@@ -897,7 +916,7 @@
       <c r="K18" s="20"/>
     </row>
     <row r="19" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="21"/>
+      <c r="B19" s="6"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -905,7 +924,8 @@
       <c r="G19" s="10"/>
       <c r="H19" s="19"/>
       <c r="I19" s="6"/>
-      <c r="J19" s="21"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="20"/>
     </row>
     <row r="20" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="21"/>
@@ -11697,6 +11717,17 @@
       <c r="H1000" s="19"/>
       <c r="I1000" s="6"/>
       <c r="J1000" s="21"/>
+    </row>
+    <row r="1001" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1001" s="21"/>
+      <c r="C1001" s="6"/>
+      <c r="D1001" s="6"/>
+      <c r="E1001" s="6"/>
+      <c r="F1001" s="14"/>
+      <c r="G1001" s="10"/>
+      <c r="H1001" s="19"/>
+      <c r="I1001" s="6"/>
+      <c r="J1001" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -11724,7 +11755,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>0</v>
@@ -11736,7 +11767,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>4</v>
@@ -11770,28 +11801,28 @@
     </row>
     <row r="2" spans="1:27" ht="96" x14ac:dyDescent="0.2">
       <c r="A2" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B2" s="6">
         <v>1</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>13</v>
@@ -11817,25 +11848,25 @@
     </row>
     <row r="3" spans="1:27" ht="80" x14ac:dyDescent="0.2">
       <c r="A3" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" s="6">
         <v>2</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="E3" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H3" s="6" t="s">
         <v>16</v>
@@ -11862,51 +11893,51 @@
     </row>
     <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B4" s="6">
         <v>3</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
     </row>
     <row r="5" spans="1:27" ht="80" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B5" s="6">
         <v>4</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="E5" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I5" s="6"/>
     </row>

</xml_diff>

<commit_message>
fix(similarity): Mention all copied columns in amdt comment prefix
</commit_message>
<xml_diff>
--- a/tests/integration/test_data/test_similarities_body.xlsx
+++ b/tests/integration/test_data/test_similarities_body.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Vidy/code/dnum/graal/tests/integration/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6EFAEE4-A606-6B44-9DCB-9F717B38196E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC31FC3B-F546-DB40-AA01-0DE61BD2046E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="28300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="vieux amendements" sheetId="1" r:id="rId1"/>
@@ -133,14 +133,13 @@
     <t>PLFSS 2024</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2024
-Numéro d'amendement : 4
-Lecture : an 16
-Organe : Organe456
-Colonne similaire : Corps amdt</t>
+    <t>DIFFERENT PROJECT</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2024
+    <t>MAUVAIS ARTICLE</t>
+  </si>
+  <si>
+    <t>Copie de Réponse, Sort depuis : PLFSS 2024
 Numéro d'amendement : 2
 Lecture : an 16
 Organe : Organe123
@@ -148,17 +147,18 @@
 Sort copié : Irrecevable</t>
   </si>
   <si>
-    <t>Réponse copiée de : PLFSS 2024
+    <t>Copie de Réponse, Sort depuis : PLFSS 2024
 Numéro d'amendement : 3
 Lecture : an 17
 Organe : Organe234
 Colonne similaire : Corps amdt</t>
   </si>
   <si>
-    <t>DIFFERENT PROJECT</t>
-  </si>
-  <si>
-    <t>MAUVAIS ARTICLE</t>
+    <t>Copie de Réponse, Sort depuis : PLFSS 2024
+Numéro d'amendement : 4
+Lecture : an 16
+Organe : Organe456
+Colonne similaire : Corps amdt</t>
   </si>
 </sst>
 </file>
@@ -704,7 +704,7 @@
     </row>
     <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B5" s="6">
         <v>3</v>
@@ -774,7 +774,7 @@
         <v>9</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>15</v>
@@ -11813,7 +11813,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>23</v>
@@ -11860,7 +11860,7 @@
         <v>21</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>23</v>
@@ -11928,7 +11928,7 @@
         <v>21</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>23</v>

</xml_diff>